<commit_message>
Merge updated Annual Plan section into the BRD and renumber
- Section 4.4 is now Annual Plan only, with the reviewer's updated use
  cases (old UC22 merged into UC19, old UC24 into the budget operations
  use case) and screenshots
- Endowment and plan-linking use cases move to a new section 4.5
- Renumber use cases (UC01-UC94), sections, BRQ001-BRQ847 and
  ERR001-ERR197, updating all cross-references; drop an empty and a
  duplicate requirement row
- Regenerate the use-case status tracker

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRM7gnnA9AXrzoXHdE9dQs
</commit_message>
<xml_diff>
--- a/docs/business-analysis/uc-status.xlsx
+++ b/docs/business-analysis/uc-status.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'UC Status'!$A$1:$E$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'UC Status'!$A$1:$E$95</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E97"/>
+  <dimension ref="A1:E95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -999,7 +999,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>UC19 – Browse the annual plans portfolio</t>
+          <t>UC19 – View and Monitor Annual Plans</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1019,14 +1019,14 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Annual Plan, Budget &amp; Endowments</t>
+          <t>Annual Plan</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>UC20 – Create an annual plan</t>
+          <t>UC20 – Create an Annual Plan</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1046,14 +1046,14 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Annual Plan, Budget &amp; Endowments</t>
+          <t>Annual Plan</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>UC21 – Build, restructure and approve a plan in an evidenced edit session</t>
+          <t>UC21 – Edit and Approve an Annual Plan</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1073,14 +1073,14 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Annual Plan, Budget &amp; Endowments</t>
+          <t>Annual Plan</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>UC22 – Monitor plan budget performance</t>
+          <t>UC22 – Manage Budget Operations and History</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1100,14 +1100,14 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Annual Plan, Budget &amp; Endowments</t>
+          <t>Annual Plan</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>UC23 – Adjust a plan budget (increase, decrease or transfer)</t>
+          <t>UC23 – Lock or Reopen an Annual Plan</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1127,14 +1127,14 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Annual Plan, Budget &amp; Endowments</t>
+          <t>Annual Plan</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>UC24 – Review financial operations and plan change history</t>
+          <t>UC24 – Record endowment funding</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1149,19 +1149,19 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>4.4.6</t>
+          <t>4.5.1</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Annual Plan, Budget &amp; Endowments</t>
+          <t>Endowments and Plan Funding Links</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>UC25 – Lock and reopen a plan budget</t>
+          <t>UC25 – Manage endowment participation and review endowment share</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1176,19 +1176,19 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>4.4.7</t>
+          <t>4.5.2</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Annual Plan, Budget &amp; Endowments</t>
+          <t>Endowments and Plan Funding Links</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>UC26 – Record endowment funding</t>
+          <t>UC26 – Link applications, projects and opportunities to plan items</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1203,19 +1203,19 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>4.4.8</t>
+          <t>4.5.3</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Annual Plan, Budget &amp; Endowments</t>
+          <t>Endowments and Plan Funding Links</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>UC27 – Manage endowment participation and review endowment share</t>
+          <t>UC27 – Monitor the grant opportunities portfolio and performance</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1230,19 +1230,19 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>4.4.9</t>
+          <t>4.6.1</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Annual Plan, Budget &amp; Endowments</t>
+          <t>Grant Opportunities, Products &amp; Workflow Templates</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>UC28 – Link applications, projects and opportunities to plan items</t>
+          <t>UC28 – Create a grant opportunity</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1257,19 +1257,19 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>4.4.10</t>
+          <t>4.6.2</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Annual Plan, Budget &amp; Endowments</t>
+          <t>Grant Opportunities, Products &amp; Workflow Templates</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>UC29 – Monitor the grant opportunities portfolio and performance</t>
+          <t>UC29 – Maintain opportunity information, reception window and status</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>4.5.1</t>
+          <t>4.6.3</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1296,7 +1296,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>UC30 – Create a grant opportunity</t>
+          <t>UC30 – Define eligibility targeting and application quota</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>4.5.2</t>
+          <t>4.6.4</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -1323,7 +1323,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>UC31 – Maintain opportunity information, reception window and status</t>
+          <t>UC31 – Configure the opportunity workflow, evaluation, form and post-approval defaults</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>4.5.3</t>
+          <t>4.6.5</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1350,7 +1350,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>UC32 – Define eligibility targeting and application quota</t>
+          <t>UC32 – Manage workflow templates and apply them to opportunities</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>4.5.4</t>
+          <t>4.6.6</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1377,7 +1377,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>UC33 – Configure the opportunity workflow, evaluation, form and post-approval defaults</t>
+          <t>UC33 – Manage the product catalog and product grant opportunities</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>4.5.5</t>
+          <t>4.6.7</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1404,7 +1404,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>UC34 – Manage workflow templates and apply them to opportunities</t>
+          <t>UC34 – Invite targeted partners to an opportunity</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>4.5.6</t>
+          <t>4.6.8</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -1431,7 +1431,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>UC35 – Manage the product catalog and product grant opportunities</t>
+          <t>UC35 – Define a tendered project (RFP) and award it to the best offer</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>4.5.7</t>
+          <t>4.6.9</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -1458,7 +1458,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>UC36 – Invite targeted partners to an opportunity</t>
+          <t>UC36 – Govern configuration changes with evidence, rollback and history</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>4.5.8</t>
+          <t>4.6.10</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -1485,7 +1485,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>UC37 – Define a tendered project (RFP) and award it to the best offer</t>
+          <t>UC37 – Self-register a partner organization</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1500,19 +1500,19 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>4.5.9</t>
+          <t>4.7.1</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Grant Opportunities, Products &amp; Workflow Templates</t>
+          <t>Partner Portal &amp; Grant Application</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>UC38 – Govern configuration changes with evidence, rollback and history</t>
+          <t>UC38 – Join a registered organization or request a delegate change</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -1527,19 +1527,19 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>4.5.10</t>
+          <t>4.7.2</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Grant Opportunities, Products &amp; Workflow Templates</t>
+          <t>Partner Portal &amp; Grant Application</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>UC39 – Self-register a partner organization</t>
+          <t>UC39 – Access the partner portal and select the represented organization</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>4.6.1</t>
+          <t>4.7.3</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -1566,7 +1566,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>UC40 – Join a registered organization or request a delegate change</t>
+          <t>UC40 – Discover open grant opportunities and check eligibility</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>4.6.2</t>
+          <t>4.7.4</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -1593,7 +1593,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>UC41 – Access the partner portal and select the represented organization</t>
+          <t>UC41 – Respond to a private opportunity invitation</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>4.6.3</t>
+          <t>4.7.5</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -1620,7 +1620,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>UC42 – Discover open grant opportunities and check eligibility</t>
+          <t>UC42 – Prepare and submit a grant application</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>4.6.4</t>
+          <t>4.7.6</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -1647,7 +1647,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>UC43 – Respond to a private opportunity invitation</t>
+          <t>UC43 – Track applications and respond to grantor requests</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>4.6.5</t>
+          <t>4.7.7</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -1674,7 +1674,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>UC44 – Prepare and submit a grant application</t>
+          <t>UC44 – Maintain the organization profile</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -1689,7 +1689,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>4.6.6</t>
+          <t>4.7.8</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -1701,7 +1701,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>UC45 – Track applications and respond to grantor requests</t>
+          <t>UC45 – Participate in project execution and confirm payment receipt</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -1716,7 +1716,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>4.6.7</t>
+          <t>4.7.9</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -1728,7 +1728,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>UC46 – Maintain the organization profile</t>
+          <t>UC46 – Receive an external AI evaluation report for an application</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>4.6.8</t>
+          <t>4.7.10</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -1755,7 +1755,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>UC47 – Participate in project execution and confirm payment receipt</t>
+          <t>UC47 – Review and decide a partner registration request</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -1770,19 +1770,19 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>4.6.9</t>
+          <t>4.8.1</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Partner Portal &amp; Grant Application</t>
+          <t>Partner Organizations Management</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>UC48 – Receive an external AI evaluation report for an application</t>
+          <t>UC48 – Browse, filter and export the partner directory</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -1797,19 +1797,19 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>4.6.10</t>
+          <t>4.8.2</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Partner Portal &amp; Grant Application</t>
+          <t>Partner Organizations Management</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>UC49 – Review and decide a partner registration request</t>
+          <t>UC49 – View the partner 360 profile and decision timeline</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -1824,7 +1824,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>4.7.1</t>
+          <t>4.8.3</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -1836,7 +1836,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>UC50 – Browse, filter and export the partner directory</t>
+          <t>UC50 – Confirm or block a partner organization</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>4.7.2</t>
+          <t>4.8.4</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -1863,7 +1863,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>UC51 – View the partner 360 profile and decision timeline</t>
+          <t>UC51 – Verify or reject a partner bank account</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -1878,7 +1878,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>4.7.3</t>
+          <t>4.8.5</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -1890,7 +1890,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>UC52 – Confirm or block a partner organization</t>
+          <t>UC52 – Review a partner license and official data update</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>4.7.4</t>
+          <t>4.8.6</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -1917,7 +1917,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>UC53 – Verify or reject a partner bank account</t>
+          <t>UC53 – Manage the partner team and primary delegate</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -1932,7 +1932,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>4.7.5</t>
+          <t>4.8.7</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -1944,7 +1944,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>UC54 – Review a partner license and official data update</t>
+          <t>UC54 – Invite a partner to activate its account</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>4.7.6</t>
+          <t>4.8.8</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -1971,7 +1971,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>UC55 – Manage the partner team and primary delegate</t>
+          <t>UC55 – Add a partner organization manually</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>4.7.7</t>
+          <t>4.8.9</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -1998,7 +1998,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>UC56 – Invite a partner to activate its account</t>
+          <t>UC56 – Manage partner groups for opportunity targeting</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -2013,7 +2013,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>4.7.8</t>
+          <t>4.8.10</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -2025,7 +2025,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>UC57 – Add a partner organization manually</t>
+          <t>UC57 – Manage the grant applications review queue</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2040,19 +2040,19 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>4.7.9</t>
+          <t>4.9.1</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Partner Organizations Management</t>
+          <t>Application Review, Evaluation &amp; Decision</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>UC58 – Manage partner groups for opportunity targeting</t>
+          <t>UC58 – Study the application dossier and its audit trail</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -2067,19 +2067,19 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>4.7.10</t>
+          <t>4.9.2</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Partner Organizations Management</t>
+          <t>Application Review, Evaluation &amp; Decision</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>UC59 – Manage the grant applications review queue</t>
+          <t>UC59 – Evaluate an application with AI decision support</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2094,7 +2094,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>4.8.1</t>
+          <t>4.9.3</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -2106,7 +2106,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>UC60 – Study the application dossier and its audit trail</t>
+          <t>UC60 – Take a stage decision on an application</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>4.8.2</t>
+          <t>4.9.4</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -2133,7 +2133,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>UC61 – Evaluate an application with AI decision support</t>
+          <t>UC61 – Return an application to the partner for edits or revised figures</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -2148,7 +2148,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>4.8.3</t>
+          <t>4.9.5</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -2160,7 +2160,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>UC62 – Take a stage decision on an application</t>
+          <t>UC62 – Record a committee decision by minute</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>4.8.4</t>
+          <t>4.9.6</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -2187,7 +2187,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>UC63 – Return an application to the partner for edits or revised figures</t>
+          <t>UC63 – Set funding conditions, indicators and initiative placement</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>4.8.5</t>
+          <t>4.9.7</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -2214,7 +2214,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>UC64 – Record a committee decision by minute</t>
+          <t>UC64 – Merge and unmerge applications of the same partner</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>4.8.6</t>
+          <t>4.9.8</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -2241,7 +2241,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>UC65 – Set funding conditions, indicators and initiative placement</t>
+          <t>UC65 – Approve the contract and transfer an approved application to projects</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>4.8.7</t>
+          <t>4.9.9</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -2268,7 +2268,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>UC66 – Merge and unmerge applications of the same partner</t>
+          <t>UC66 – Approve and deliver an in-kind (product) grant</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>4.8.8</t>
+          <t>4.9.10</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -2295,7 +2295,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>UC67 – Approve the contract and transfer an approved application to projects</t>
+          <t>UC67 – Prepare the bill of quantities and payment schedule</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -2310,19 +2310,19 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>4.8.9</t>
+          <t>4.10.1</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Application Review, Evaluation &amp; Decision</t>
+          <t>Projects, Contracts &amp; Execution Monitoring</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>UC68 – Approve and deliver an in-kind (product) grant</t>
+          <t>UC68 – Approve the contract and transfer the application into project(s)</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -2337,19 +2337,19 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>4.8.10</t>
+          <t>4.10.2</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Application Review, Evaluation &amp; Decision</t>
+          <t>Projects, Contracts &amp; Execution Monitoring</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>UC69 – Prepare the bill of quantities and payment schedule</t>
+          <t>UC69 – Manage contract signing and the contracts register</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>4.9.1</t>
+          <t>4.10.3</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -2376,7 +2376,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>UC70 – Approve the contract and transfer the application into project(s)</t>
+          <t>UC70 – Monitor the project portfolio and project status</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -2391,7 +2391,7 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>4.9.2</t>
+          <t>4.10.4</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -2403,7 +2403,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>UC71 – Manage contract signing and the contracts register</t>
+          <t>UC71 – Create an internal initiative</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>4.9.3</t>
+          <t>4.10.5</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -2430,7 +2430,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>UC72 – Monitor the project portfolio and project status</t>
+          <t>UC72 – Plan the project and start execution</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>4.9.4</t>
+          <t>4.10.6</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
@@ -2457,7 +2457,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>UC73 – Create an internal initiative</t>
+          <t>UC73 – Execute tasks and report progress</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>4.9.5</t>
+          <t>4.10.7</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -2484,7 +2484,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>UC74 – Plan the project and start execution</t>
+          <t>UC74 – Verify work and approve milestones</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -2499,7 +2499,7 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>4.9.6</t>
+          <t>4.10.8</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
@@ -2511,7 +2511,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>UC75 – Execute tasks and report progress</t>
+          <t>UC75 – Request and approve a plan revision</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>4.9.7</t>
+          <t>4.10.9</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -2538,7 +2538,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>UC76 – Verify work and approve milestones</t>
+          <t>UC76 – Close the project and confirm results</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>4.9.8</t>
+          <t>4.10.10</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
@@ -2565,7 +2565,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>UC77 – Request and approve a plan revision</t>
+          <t>UC77 – Monitor the payments register</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -2580,19 +2580,19 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>4.9.9</t>
+          <t>4.11.1</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Projects, Contracts &amp; Execution Monitoring</t>
+          <t>Payments, Disbursement &amp; Financial Reporting</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>UC78 – Close the project and confirm results</t>
+          <t>UC78 – Make a payment due and submit it for approval</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -2607,19 +2607,19 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>4.9.10</t>
+          <t>4.11.2</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Projects, Contracts &amp; Execution Monitoring</t>
+          <t>Payments, Disbursement &amp; Financial Reporting</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>UC79 – Monitor the payments register</t>
+          <t>UC79 – Approve or reject a payment</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>4.10.1</t>
+          <t>4.11.3</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -2646,7 +2646,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>UC80 – Make a payment due and submit it for approval</t>
+          <t>UC80 – Issue the disbursement order and confirm the payee</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -2661,7 +2661,7 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>4.10.2</t>
+          <t>4.11.4</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
@@ -2673,7 +2673,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>UC81 – Approve or reject a payment</t>
+          <t>UC81 – Record the bank transfer</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -2688,7 +2688,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>4.10.3</t>
+          <t>4.11.5</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -2700,7 +2700,7 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>UC82 – Issue the disbursement order and confirm the payee</t>
+          <t>UC82 – Confirm receipt and close the payment</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>4.10.4</t>
+          <t>4.11.6</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
@@ -2727,7 +2727,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>UC83 – Record the bank transfer</t>
+          <t>UC83 – Monitor financial position and partner commitments</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -2742,7 +2742,7 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>4.10.5</t>
+          <t>4.11.7</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -2754,7 +2754,7 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>UC84 – Confirm receipt and close the payment</t>
+          <t>UC84 – View the executive indicators dashboard</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -2769,7 +2769,7 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>4.10.6</t>
+          <t>4.11.8</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
@@ -2781,7 +2781,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>UC85 – Monitor financial position and partner commitments</t>
+          <t>UC85 – Produce operational and financial reports</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>4.10.7</t>
+          <t>4.11.9</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -2808,7 +2808,7 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>UC86 – View the executive indicators dashboard</t>
+          <t>UC86 – Receive application stage tasks automatically</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -2823,19 +2823,19 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>4.10.8</t>
+          <t>4.12.1</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Payments, Disbursement &amp; Financial Reporting</t>
+          <t>Work Management &amp; Tasks</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>UC87 – Produce operational and financial reports</t>
+          <t>UC87 – Receive payment approval and execution tasks</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -2850,19 +2850,19 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>4.10.9</t>
+          <t>4.12.2</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Payments, Disbursement &amp; Financial Reporting</t>
+          <t>Work Management &amp; Tasks</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>UC88 – Receive application stage tasks automatically</t>
+          <t>UC88 – Organise and monitor my work inbox</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -2877,7 +2877,7 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>4.11.1</t>
+          <t>4.12.3</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -2889,7 +2889,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>UC89 – Receive payment approval and execution tasks</t>
+          <t>UC89 – Create, assign and edit a manual task</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -2904,7 +2904,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>4.11.2</t>
+          <t>4.12.4</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -2916,7 +2916,7 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>UC90 – Organise and monitor my work inbox</t>
+          <t>UC90 – Schedule a meeting</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>4.11.3</t>
+          <t>4.12.5</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -2943,7 +2943,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>UC91 – Create, assign and edit a manual task</t>
+          <t>UC91 – Track progress and close a manual task</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -2958,7 +2958,7 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>4.11.4</t>
+          <t>4.12.6</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -2970,7 +2970,7 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>UC92 – Schedule a meeting</t>
+          <t>UC92 – Take a decision directly from a task</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>4.11.5</t>
+          <t>4.12.7</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -2997,7 +2997,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>UC93 – Track progress and close a manual task</t>
+          <t>UC93 – Decide several committee items with one minute</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -3012,7 +3012,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>4.11.6</t>
+          <t>4.12.8</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -3024,7 +3024,7 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>UC94 – Take a decision directly from a task</t>
+          <t>UC94 – Process tasks in focus mode</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>4.11.7</t>
+          <t>4.12.9</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -3048,62 +3048,8 @@
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="2" t="inlineStr">
-        <is>
-          <t>UC95 – Decide several committee items with one minute</t>
-        </is>
-      </c>
-      <c r="B96" s="2" t="inlineStr">
-        <is>
-          <t>UC95</t>
-        </is>
-      </c>
-      <c r="C96" s="5" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="D96" s="2" t="inlineStr">
-        <is>
-          <t>4.11.8</t>
-        </is>
-      </c>
-      <c r="E96" s="2" t="inlineStr">
-        <is>
-          <t>Work Management &amp; Tasks</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="2" t="inlineStr">
-        <is>
-          <t>UC96 – Process tasks in focus mode</t>
-        </is>
-      </c>
-      <c r="B97" s="2" t="inlineStr">
-        <is>
-          <t>UC96</t>
-        </is>
-      </c>
-      <c r="C97" s="5" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="D97" s="2" t="inlineStr">
-        <is>
-          <t>4.11.9</t>
-        </is>
-      </c>
-      <c r="E97" s="2" t="inlineStr">
-        <is>
-          <t>Work Management &amp; Tasks</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E97"/>
+  <autoFilter ref="A1:E95"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3175,11 +3121,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>UC19–UC96</t>
+          <t>UC19–UC94</t>
         </is>
       </c>
     </row>
@@ -3190,7 +3136,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C5" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Mark annual plan use cases (UC19-UC23) as pending in the status tracker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRM7gnnA9AXrzoXHdE9dQs
</commit_message>
<xml_diff>
--- a/docs/business-analysis/uc-status.xlsx
+++ b/docs/business-analysis/uc-status.xlsx
@@ -1007,9 +1007,9 @@
           <t>UC19</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>draft</t>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1034,9 +1034,9 @@
           <t>UC20</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>draft</t>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1061,9 +1061,9 @@
           <t>UC21</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>draft</t>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1088,9 +1088,9 @@
           <t>UC22</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>draft</t>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1115,9 +1115,9 @@
           <t>UC23</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>draft</t>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -3106,11 +3106,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>UC11–UC18</t>
+          <t>UC11–UC23</t>
         </is>
       </c>
     </row>
@@ -3121,11 +3121,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>UC19–UC94</t>
+          <t>UC24–UC94</t>
         </is>
       </c>
     </row>

</xml_diff>